<commit_message>
Gage reach lookup table
</commit_message>
<xml_diff>
--- a/GageTable_All.xlsx
+++ b/GageTable_All.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\workspace\DRAFT\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{48954918-D98A-4BD6-89E8-4BF7D2E6F4F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D1A08AF-C7CE-4874-99C1-389447FF6B93}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="41200" yWindow="3140" windowWidth="28800" windowHeight="15350" xr2:uid="{537AAD5D-038D-4158-A401-D053F9117A77}"/>
+    <workbookView xWindow="38310" yWindow="20" windowWidth="19380" windowHeight="20950" xr2:uid="{537AAD5D-038D-4158-A401-D053F9117A77}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="351" uniqueCount="199">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="369" uniqueCount="221">
   <si>
     <t>Gage</t>
   </si>
@@ -617,22 +617,88 @@
     <t>CEMVR_IL_MA_MVR_26</t>
   </si>
   <si>
-    <t>CEMVR_IL_</t>
-  </si>
-  <si>
-    <t>CEMVR_UM</t>
-  </si>
-  <si>
-    <t>CEMVR_IL_MA_MVR</t>
-  </si>
-  <si>
-    <t>CEMVR_IL_PE_MVR</t>
-  </si>
-  <si>
-    <t>CEMVR_IL_SR_MVR</t>
-  </si>
-  <si>
     <t>CEMVR_IL_LA_MVR_1</t>
+  </si>
+  <si>
+    <t>CEMVR_IL_MA_MVR_1</t>
+  </si>
+  <si>
+    <t>CEMVR_IL_SR_MVR_1</t>
+  </si>
+  <si>
+    <t>CEMVR_IL_PE_MVR_1</t>
+  </si>
+  <si>
+    <t>CEMVR_UM_11_MVR_31</t>
+  </si>
+  <si>
+    <t>CEMVR_UM_12_MVR_1</t>
+  </si>
+  <si>
+    <t>CEMVR_UM_12_MVR_26</t>
+  </si>
+  <si>
+    <t>CEMVR_UM_13_MVR_1</t>
+  </si>
+  <si>
+    <t>CEMVR_UM_13_MVR_33</t>
+  </si>
+  <si>
+    <t>CEMVR_UM_14_MVR_1</t>
+  </si>
+  <si>
+    <t>CEMVR_UM_14_MVR_28</t>
+  </si>
+  <si>
+    <t>CEMVR_UM_15_MVR_1</t>
+  </si>
+  <si>
+    <t>CEMVR_UM_15_MVR_10</t>
+  </si>
+  <si>
+    <t>CEMVR_UM_16_MVR_1</t>
+  </si>
+  <si>
+    <t>CEMVR_UM_16_MVR_26</t>
+  </si>
+  <si>
+    <t>CEMVR_UM_17_MVR_1</t>
+  </si>
+  <si>
+    <t>CEMVR_UM_17_MVR_20</t>
+  </si>
+  <si>
+    <t>CEMVR_UM_18_MVR_1</t>
+  </si>
+  <si>
+    <t>CEMVR_UM_19_MVR_1</t>
+  </si>
+  <si>
+    <t>CEMVR_UM_20_MVR_20</t>
+  </si>
+  <si>
+    <t>CEMVR_UM_20_MVR_1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CEMVR_UM_21_MVR_1 </t>
+  </si>
+  <si>
+    <t>CEMVR_UM_22_MVR_1</t>
+  </si>
+  <si>
+    <t>CEMVR_UM_18_MVR_26</t>
+  </si>
+  <si>
+    <t>CEMVR_UM_19_MVR_46</t>
+  </si>
+  <si>
+    <t>CEMVR_UM_21_MVR_18</t>
+  </si>
+  <si>
+    <t>CEMVR_UM_22_MVR_24</t>
+  </si>
+  <si>
+    <t>CEMVR_UM_24_MVR_1</t>
   </si>
 </sst>
 </file>
@@ -1058,16 +1124,16 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F0574D8B-9E50-40DF-8B17-DB7E83DDCAFC}">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:L68"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
-    <col min="1" max="1" width="11.26953125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="32.81640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.6328125" style="1" customWidth="1"/>
-    <col min="5" max="6" width="10.90625" customWidth="1"/>
-    <col min="7" max="7" width="19.54296875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.26171875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="32.7890625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.62890625" style="1" customWidth="1"/>
+    <col min="5" max="6" width="10.89453125" customWidth="1"/>
+    <col min="7" max="7" width="19.5234375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1090,7 +1156,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.55000000000000004">
       <c r="A2" s="1" t="s">
         <v>165</v>
       </c>
@@ -1102,7 +1168,7 @@
       </c>
       <c r="H2" s="1"/>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.55000000000000004">
       <c r="A3" s="1" t="s">
         <v>163</v>
       </c>
@@ -1114,7 +1180,7 @@
       </c>
       <c r="H3" s="1"/>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.55000000000000004">
       <c r="A4" s="1" t="s">
         <v>162</v>
       </c>
@@ -1126,7 +1192,7 @@
       </c>
       <c r="H4" s="1"/>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.55000000000000004">
       <c r="A5" s="1" t="s">
         <v>152</v>
       </c>
@@ -1135,7 +1201,7 @@
       </c>
       <c r="H5" s="1"/>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.55000000000000004">
       <c r="A6" s="1" t="s">
         <v>166</v>
       </c>
@@ -1147,7 +1213,7 @@
       </c>
       <c r="H6" s="1"/>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.55000000000000004">
       <c r="A7" s="1" t="s">
         <v>158</v>
       </c>
@@ -1159,7 +1225,7 @@
       </c>
       <c r="H7" s="1"/>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.55000000000000004">
       <c r="A8" s="1" t="s">
         <v>164</v>
       </c>
@@ -1171,7 +1237,7 @@
       </c>
       <c r="H8" s="1"/>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.55000000000000004">
       <c r="A9" t="s">
         <v>3</v>
       </c>
@@ -1192,7 +1258,7 @@
       </c>
       <c r="H9" s="1"/>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.55000000000000004">
       <c r="A10" t="s">
         <v>4</v>
       </c>
@@ -1213,7 +1279,7 @@
       </c>
       <c r="H10" s="1"/>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.55000000000000004">
       <c r="A11" t="s">
         <v>5</v>
       </c>
@@ -1234,7 +1300,7 @@
       </c>
       <c r="H11" s="1"/>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.55000000000000004">
       <c r="A12" t="s">
         <v>6</v>
       </c>
@@ -1255,7 +1321,7 @@
       </c>
       <c r="H12" s="1"/>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.55000000000000004">
       <c r="A13" t="s">
         <v>7</v>
       </c>
@@ -1276,7 +1342,7 @@
       </c>
       <c r="H13" s="1"/>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.55000000000000004">
       <c r="A14" t="s">
         <v>8</v>
       </c>
@@ -1297,7 +1363,7 @@
       </c>
       <c r="H14" s="1"/>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.55000000000000004">
       <c r="A15" t="s">
         <v>9</v>
       </c>
@@ -1318,7 +1384,7 @@
       </c>
       <c r="H15" s="1"/>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.55000000000000004">
       <c r="A16" t="s">
         <v>10</v>
       </c>
@@ -1339,7 +1405,7 @@
       </c>
       <c r="H16" s="1"/>
     </row>
-    <row r="17" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:12" x14ac:dyDescent="0.55000000000000004">
       <c r="A17" t="s">
         <v>11</v>
       </c>
@@ -1369,7 +1435,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="18" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:12" x14ac:dyDescent="0.55000000000000004">
       <c r="A18" t="s">
         <v>12</v>
       </c>
@@ -1399,7 +1465,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="19" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:12" x14ac:dyDescent="0.55000000000000004">
       <c r="A19" t="s">
         <v>13</v>
       </c>
@@ -1429,7 +1495,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="20" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:12" x14ac:dyDescent="0.55000000000000004">
       <c r="A20" t="s">
         <v>14</v>
       </c>
@@ -1459,7 +1525,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="21" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:12" x14ac:dyDescent="0.55000000000000004">
       <c r="A21" t="s">
         <v>15</v>
       </c>
@@ -1489,7 +1555,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="22" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:12" x14ac:dyDescent="0.55000000000000004">
       <c r="A22" t="s">
         <v>16</v>
       </c>
@@ -1519,7 +1585,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="23" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:12" x14ac:dyDescent="0.55000000000000004">
       <c r="A23" t="s">
         <v>17</v>
       </c>
@@ -1536,7 +1602,7 @@
         <v>126</v>
       </c>
       <c r="G23" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="H23" s="1"/>
       <c r="J23" s="5" t="s">
@@ -1549,7 +1615,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="24" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:12" x14ac:dyDescent="0.55000000000000004">
       <c r="A24" t="s">
         <v>18</v>
       </c>
@@ -1566,7 +1632,7 @@
         <v>126</v>
       </c>
       <c r="G24" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="H24" s="1"/>
       <c r="J24" s="5" t="s">
@@ -1579,7 +1645,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="25" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:12" x14ac:dyDescent="0.55000000000000004">
       <c r="A25" t="s">
         <v>19</v>
       </c>
@@ -1596,7 +1662,7 @@
         <v>126</v>
       </c>
       <c r="G25" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="H25" s="1"/>
       <c r="J25" s="5" t="s">
@@ -1609,7 +1675,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="26" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:12" x14ac:dyDescent="0.55000000000000004">
       <c r="A26" t="s">
         <v>20</v>
       </c>
@@ -1626,7 +1692,7 @@
         <v>126</v>
       </c>
       <c r="G26" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="H26" s="1"/>
       <c r="J26" s="5" t="s">
@@ -1639,7 +1705,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="27" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:12" x14ac:dyDescent="0.55000000000000004">
       <c r="A27" t="s">
         <v>21</v>
       </c>
@@ -1669,7 +1735,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="28" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:12" x14ac:dyDescent="0.55000000000000004">
       <c r="A28" t="s">
         <v>22</v>
       </c>
@@ -1696,7 +1762,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="29" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:12" x14ac:dyDescent="0.55000000000000004">
       <c r="A29" t="s">
         <v>23</v>
       </c>
@@ -1713,7 +1779,7 @@
         <v>126</v>
       </c>
       <c r="G29" t="s">
-        <v>198</v>
+        <v>193</v>
       </c>
       <c r="H29" s="1"/>
       <c r="J29" s="5" t="s">
@@ -1723,7 +1789,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="30" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:12" x14ac:dyDescent="0.55000000000000004">
       <c r="A30" t="s">
         <v>24</v>
       </c>
@@ -1738,6 +1804,9 @@
       </c>
       <c r="E30" t="s">
         <v>126</v>
+      </c>
+      <c r="G30" t="s">
+        <v>193</v>
       </c>
       <c r="H30" s="1"/>
       <c r="J30" s="5" t="s">
@@ -1747,7 +1816,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="31" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:12" x14ac:dyDescent="0.55000000000000004">
       <c r="A31" t="s">
         <v>25</v>
       </c>
@@ -1774,7 +1843,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="32" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:12" x14ac:dyDescent="0.55000000000000004">
       <c r="A32" t="s">
         <v>26</v>
       </c>
@@ -1801,7 +1870,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="33" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:11" x14ac:dyDescent="0.55000000000000004">
       <c r="A33" t="s">
         <v>27</v>
       </c>
@@ -1828,7 +1897,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="34" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:11" x14ac:dyDescent="0.55000000000000004">
       <c r="A34" t="s">
         <v>28</v>
       </c>
@@ -1844,9 +1913,12 @@
       <c r="E34" t="s">
         <v>126</v>
       </c>
+      <c r="G34" t="s">
+        <v>197</v>
+      </c>
       <c r="H34" s="1"/>
     </row>
-    <row r="35" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:11" x14ac:dyDescent="0.55000000000000004">
       <c r="A35" t="s">
         <v>29</v>
       </c>
@@ -1862,9 +1934,12 @@
       <c r="E35" t="s">
         <v>126</v>
       </c>
+      <c r="G35" t="s">
+        <v>198</v>
+      </c>
       <c r="H35" s="1"/>
     </row>
-    <row r="36" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:11" x14ac:dyDescent="0.55000000000000004">
       <c r="A36" t="s">
         <v>30</v>
       </c>
@@ -1880,9 +1955,12 @@
       <c r="E36" t="s">
         <v>126</v>
       </c>
+      <c r="G36" t="s">
+        <v>199</v>
+      </c>
       <c r="H36" s="1"/>
     </row>
-    <row r="37" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:11" x14ac:dyDescent="0.55000000000000004">
       <c r="A37" t="s">
         <v>31</v>
       </c>
@@ -1898,9 +1976,12 @@
       <c r="E37" t="s">
         <v>126</v>
       </c>
+      <c r="G37" t="s">
+        <v>200</v>
+      </c>
       <c r="H37" s="1"/>
     </row>
-    <row r="38" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:11" x14ac:dyDescent="0.55000000000000004">
       <c r="A38" t="s">
         <v>32</v>
       </c>
@@ -1916,9 +1997,12 @@
       <c r="E38" t="s">
         <v>126</v>
       </c>
+      <c r="G38" t="s">
+        <v>201</v>
+      </c>
       <c r="H38" s="1"/>
     </row>
-    <row r="39" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:11" x14ac:dyDescent="0.55000000000000004">
       <c r="A39" t="s">
         <v>33</v>
       </c>
@@ -1934,9 +2018,12 @@
       <c r="E39" t="s">
         <v>126</v>
       </c>
+      <c r="G39" t="s">
+        <v>202</v>
+      </c>
       <c r="H39" s="1"/>
     </row>
-    <row r="40" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:11" x14ac:dyDescent="0.55000000000000004">
       <c r="A40" t="s">
         <v>34</v>
       </c>
@@ -1952,9 +2039,12 @@
       <c r="E40" t="s">
         <v>126</v>
       </c>
+      <c r="G40" t="s">
+        <v>203</v>
+      </c>
       <c r="H40" s="1"/>
     </row>
-    <row r="41" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:11" x14ac:dyDescent="0.55000000000000004">
       <c r="A41" t="s">
         <v>35</v>
       </c>
@@ -1970,9 +2060,12 @@
       <c r="E41" t="s">
         <v>126</v>
       </c>
+      <c r="G41" t="s">
+        <v>204</v>
+      </c>
       <c r="H41" s="1"/>
     </row>
-    <row r="42" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:11" x14ac:dyDescent="0.55000000000000004">
       <c r="A42" t="s">
         <v>36</v>
       </c>
@@ -1988,9 +2081,12 @@
       <c r="E42" t="s">
         <v>126</v>
       </c>
+      <c r="G42" t="s">
+        <v>205</v>
+      </c>
       <c r="H42" s="1"/>
     </row>
-    <row r="43" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:11" x14ac:dyDescent="0.55000000000000004">
       <c r="A43" t="s">
         <v>37</v>
       </c>
@@ -2006,9 +2102,12 @@
       <c r="E43" t="s">
         <v>126</v>
       </c>
+      <c r="G43" t="s">
+        <v>206</v>
+      </c>
       <c r="H43" s="1"/>
     </row>
-    <row r="44" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:11" x14ac:dyDescent="0.55000000000000004">
       <c r="A44" t="s">
         <v>38</v>
       </c>
@@ -2024,9 +2123,12 @@
       <c r="E44" t="s">
         <v>126</v>
       </c>
+      <c r="G44" t="s">
+        <v>207</v>
+      </c>
       <c r="H44" s="1"/>
     </row>
-    <row r="45" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:11" x14ac:dyDescent="0.55000000000000004">
       <c r="A45" t="s">
         <v>39</v>
       </c>
@@ -2042,9 +2144,12 @@
       <c r="E45" t="s">
         <v>126</v>
       </c>
+      <c r="G45" t="s">
+        <v>208</v>
+      </c>
       <c r="H45" s="1"/>
     </row>
-    <row r="46" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:11" x14ac:dyDescent="0.55000000000000004">
       <c r="A46" t="s">
         <v>40</v>
       </c>
@@ -2060,9 +2165,12 @@
       <c r="E46" t="s">
         <v>126</v>
       </c>
+      <c r="G46" t="s">
+        <v>209</v>
+      </c>
       <c r="H46" s="1"/>
     </row>
-    <row r="47" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:11" x14ac:dyDescent="0.55000000000000004">
       <c r="A47" t="s">
         <v>41</v>
       </c>
@@ -2078,9 +2186,12 @@
       <c r="E47" t="s">
         <v>126</v>
       </c>
+      <c r="G47" t="s">
+        <v>210</v>
+      </c>
       <c r="H47" s="1"/>
     </row>
-    <row r="48" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:11" x14ac:dyDescent="0.55000000000000004">
       <c r="A48" t="s">
         <v>42</v>
       </c>
@@ -2096,9 +2207,12 @@
       <c r="E48" t="s">
         <v>126</v>
       </c>
+      <c r="G48" t="s">
+        <v>216</v>
+      </c>
       <c r="H48" s="1"/>
     </row>
-    <row r="49" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:8" x14ac:dyDescent="0.55000000000000004">
       <c r="A49" t="s">
         <v>43</v>
       </c>
@@ -2114,9 +2228,12 @@
       <c r="E49" t="s">
         <v>126</v>
       </c>
+      <c r="G49" t="s">
+        <v>211</v>
+      </c>
       <c r="H49" s="1"/>
     </row>
-    <row r="50" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:8" x14ac:dyDescent="0.55000000000000004">
       <c r="A50" t="s">
         <v>44</v>
       </c>
@@ -2132,9 +2249,12 @@
       <c r="E50" t="s">
         <v>126</v>
       </c>
+      <c r="G50" t="s">
+        <v>217</v>
+      </c>
       <c r="H50" s="1"/>
     </row>
-    <row r="51" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:8" x14ac:dyDescent="0.55000000000000004">
       <c r="A51" t="s">
         <v>45</v>
       </c>
@@ -2150,9 +2270,12 @@
       <c r="E51" t="s">
         <v>126</v>
       </c>
+      <c r="G51" t="s">
+        <v>213</v>
+      </c>
       <c r="H51" s="1"/>
     </row>
-    <row r="52" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:8" x14ac:dyDescent="0.55000000000000004">
       <c r="A52" t="s">
         <v>46</v>
       </c>
@@ -2168,9 +2291,12 @@
       <c r="E52" t="s">
         <v>126</v>
       </c>
+      <c r="G52" t="s">
+        <v>212</v>
+      </c>
       <c r="H52" s="1"/>
     </row>
-    <row r="53" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:8" x14ac:dyDescent="0.55000000000000004">
       <c r="A53" t="s">
         <v>47</v>
       </c>
@@ -2186,9 +2312,12 @@
       <c r="E53" t="s">
         <v>126</v>
       </c>
+      <c r="G53" t="s">
+        <v>214</v>
+      </c>
       <c r="H53" s="1"/>
     </row>
-    <row r="54" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:8" x14ac:dyDescent="0.55000000000000004">
       <c r="A54" t="s">
         <v>48</v>
       </c>
@@ -2204,9 +2333,12 @@
       <c r="E54" t="s">
         <v>126</v>
       </c>
+      <c r="G54" t="s">
+        <v>218</v>
+      </c>
       <c r="H54" s="1"/>
     </row>
-    <row r="55" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:8" x14ac:dyDescent="0.55000000000000004">
       <c r="A55" t="s">
         <v>49</v>
       </c>
@@ -2222,8 +2354,11 @@
       <c r="E55" t="s">
         <v>126</v>
       </c>
-    </row>
-    <row r="56" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="G55" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="56" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A56" t="s">
         <v>50</v>
       </c>
@@ -2239,8 +2374,11 @@
       <c r="E56" t="s">
         <v>126</v>
       </c>
-    </row>
-    <row r="57" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="G56" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="57" spans="1:8" x14ac:dyDescent="0.55000000000000004">
       <c r="A57" t="s">
         <v>51</v>
       </c>
@@ -2256,8 +2394,11 @@
       <c r="E57" t="s">
         <v>126</v>
       </c>
-    </row>
-    <row r="58" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="G57" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="58" spans="1:8" x14ac:dyDescent="0.55000000000000004">
       <c r="A58" t="s">
         <v>52</v>
       </c>
@@ -2277,7 +2418,7 @@
         <v>186</v>
       </c>
     </row>
-    <row r="59" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:8" x14ac:dyDescent="0.55000000000000004">
       <c r="A59" t="s">
         <v>53</v>
       </c>
@@ -2297,7 +2438,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="60" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:8" x14ac:dyDescent="0.55000000000000004">
       <c r="A60" t="s">
         <v>54</v>
       </c>
@@ -2317,7 +2458,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="61" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:8" x14ac:dyDescent="0.55000000000000004">
       <c r="A61" t="s">
         <v>55</v>
       </c>
@@ -2337,7 +2478,7 @@
         <v>189</v>
       </c>
     </row>
-    <row r="62" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:8" x14ac:dyDescent="0.55000000000000004">
       <c r="A62" t="s">
         <v>117</v>
       </c>
@@ -2353,11 +2494,8 @@
       <c r="E62" t="s">
         <v>109</v>
       </c>
-      <c r="G62" t="s">
-        <v>194</v>
-      </c>
-    </row>
-    <row r="63" spans="1:8" x14ac:dyDescent="0.35">
+    </row>
+    <row r="63" spans="1:8" x14ac:dyDescent="0.55000000000000004">
       <c r="A63" t="s">
         <v>124</v>
       </c>
@@ -2373,11 +2511,8 @@
       <c r="E63" t="s">
         <v>109</v>
       </c>
-      <c r="G63" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="64" spans="1:8" x14ac:dyDescent="0.35">
+    </row>
+    <row r="64" spans="1:8" x14ac:dyDescent="0.55000000000000004">
       <c r="A64" t="s">
         <v>110</v>
       </c>
@@ -2393,11 +2528,8 @@
       <c r="E64" t="s">
         <v>109</v>
       </c>
-      <c r="G64" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="65" spans="1:7" x14ac:dyDescent="0.35">
+    </row>
+    <row r="65" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A65" t="s">
         <v>122</v>
       </c>
@@ -2413,11 +2545,8 @@
       <c r="E65" t="s">
         <v>109</v>
       </c>
-      <c r="G65" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="66" spans="1:7" x14ac:dyDescent="0.35">
+    </row>
+    <row r="66" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A66" t="s">
         <v>120</v>
       </c>
@@ -2433,11 +2562,8 @@
       <c r="E66" t="s">
         <v>109</v>
       </c>
-      <c r="G66" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="67" spans="1:7" x14ac:dyDescent="0.35">
+    </row>
+    <row r="67" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A67" t="s">
         <v>119</v>
       </c>
@@ -2453,11 +2579,8 @@
       <c r="E67" t="s">
         <v>109</v>
       </c>
-      <c r="G67" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="68" spans="1:7" x14ac:dyDescent="0.35">
+    </row>
+    <row r="68" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A68" t="s">
         <v>115</v>
       </c>
@@ -2472,9 +2595,6 @@
       </c>
       <c r="E68" t="s">
         <v>109</v>
-      </c>
-      <c r="G68" t="s">
-        <v>193</v>
       </c>
     </row>
   </sheetData>

</xml_diff>